<commit_message>
Implement report generation and update email forwarding logic
</commit_message>
<xml_diff>
--- a/output/email_classifications.xlsx
+++ b/output/email_classifications.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -430,11 +430,11 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
     <col width="50" customWidth="1" min="17" max="17"/>
     <col width="50" customWidth="1" min="18" max="18"/>
@@ -1120,6 +1120,426 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>edf643e0-1d30-4e44-bbe2-fd66fcde228c</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46094.38131537037</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AAMkAGIwZTNjOTA3LWVhZTUtNDI3My04NGZmLTIwMTlmY2UyZD...</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>antoni.debicki@b-yond.com</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FW: New Whitepaper Form Submission from B-Yond</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>disqualify</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Novelus</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>maroun</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>saade</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>maroun.saadeh@gmail.com</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Whitepaper name: PCAPVision: PCAP-Based High-Velocity &amp; Large-Volume NetworkFailure Detection</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>email classified successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05bc50c2-9670-402e-8588-c9c042fe3fc2</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46099.7029708912</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AAMkAGVlZDk2NTYxLWFiY2QtNDBjNS1hMTZiLThlYjE1Mjc1OT...</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>antoni.debicki@b-yond.com</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FW: New Whitepaper Form Submission from B-Yond</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>disqualify</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Novelus</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>maroun</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>saade</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>maroun.saadeh@gmail.com</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Whitepaper name: PCAPVision: PCAP-Based High-Velocity &amp; Large-Volume NetworkFailure Detection</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>email classified successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>e15363a1-11f7-4c24-a0b5-805e560bb85b</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46099.70869563657</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AAMkAGVlZDk2NTYxLWFiY2QtNDBjNS1hMTZiLThlYjE1Mjc1OT...</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>antoni.debicki@b-yond.com</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FW: New Whitepaper Form Submission from B-Yond</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>disqualify</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Novelus</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>maroun</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>saade</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>maroun.saadeh@gmail.com</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>You just received a new form submission on your website B-Yond. Whitepaper name: PCAPVision: PCAP-Ba</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>email classified successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>96d26688-1a1d-485b-acc2-6c2222b632dd</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46099.70880449074</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AAMkAGVlZDk2NTYxLWFiY2QtNDBjNS1hMTZiLThlYjE1Mjc1OT...</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>antoni.debicki@b-yond.com</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FW: New Whitepaper Form Submission from B-Yond</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>disqualify</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Novelus</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Telco Vendor</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>maroun</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>saade</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>maroun.saadeh@novelus.com</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Ziad</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Lebanon</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Lebanon, United Arab Emirates, Nigeria, Ivory Coast, Saudi Arabia, Iraq</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>5G rollout support, Cloud migration for telecom, BSS/OSS integration</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>You just received a new form submission on your website B-Yond. Whitepaper name: PCAPVision: PCAP-Ba</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>email classified successfully</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>617c4089-6561-4444-95cb-918b551e69b4</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46099.70970708333</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AAMkAGVlZDk2NTYxLWFiY2QtNDBjNS1hMTZiLThlYjE1Mjc1OT...</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>antoni.debicki@b-yond.com</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FW: New Whitepaper Form Submission from B-Yond</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>qualify</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Novelus</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Telco Vendor</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>maroun</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>saade</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>maroun.saadeh@novelus.com</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Ziad</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Lebanon, United States</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Lebanon, United States, Middle East</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Automation of network operations, Development of AI/ML solutions for networks, Network performance monitoring and optimization</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>You just received a new form submission on your website B-Yond. Whitepaper name: PCAPVision: PCAP-Ba</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>email classified successfully</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>